<commit_message>
Flux AU: portfolio names use Brand+Product convention
- "Flux Avento", "80Days StrapNylon", "80Days CL101", etc.
- Matches campaign naming convention

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/flux/20260313_Flux_AU_Portfolio_Structure.xlsx
+++ b/flux/20260313_Flux_AU_Portfolio_Structure.xlsx
@@ -488,7 +488,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-13 11:07  |  Profile: 3601686309797276  |  SP+SB Campaigns: 8734</t>
+          <t>Generated: 2026-03-13 11:25  |  Profile: 3601686309797276  |  SP+SB Campaigns: 8734</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Strap</t>
+          <t>80Days StrapNylon</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -579,7 +579,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Strap</t>
+          <t>80Days StrapWire</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -616,7 +616,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>80Days CL101</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -653,7 +653,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>80Days CL102</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -690,7 +690,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>80Days LD101</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -727,7 +727,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Avento</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -764,7 +764,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Bowrider</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -801,7 +801,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Brentwood</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -838,7 +838,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux FX21</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -875,7 +875,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Lantaka</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -912,7 +912,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Soleado</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -949,7 +949,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Sportech</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -986,7 +986,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Ventura</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1023,7 +1023,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Verano</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1168,7 +1168,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Strap</t>
+          <t>80Days StrapNylon</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1422,7 +1422,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Strap</t>
+          <t>80Days StrapWire</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1552,7 +1552,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>80Days CL101</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1632,7 +1632,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>80Days CL102</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1708,7 +1708,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>80Days LD101</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Avento</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2013,7 +2013,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Bowrider</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2122,7 +2122,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Brentwood</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux FX21</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2409,7 +2409,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Lantaka</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2518,7 +2518,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Soleado</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2596,7 +2596,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Sportech</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2788,7 +2788,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Ventura</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2984,7 +2984,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Verano</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Strap</t>
+          <t>80Days StrapNylon</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Strap</t>
+          <t>80Days StrapWire</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
@@ -3332,7 +3332,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>80Days CL101</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
@@ -3363,7 +3363,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>80Days CL102</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
@@ -3392,7 +3392,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>80Days LD101</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Avento</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Bowrider</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
@@ -3513,7 +3513,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Brentwood</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
@@ -3550,7 +3550,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux FX21</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Lantaka</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Soleado</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
@@ -3659,7 +3659,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Sportech</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Ventura</t>
         </is>
       </c>
       <c r="D16" s="4" t="n">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Verano</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Strap</t>
+          <t>80Days StrapNylon</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
@@ -3925,7 +3925,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Strap</t>
+          <t>80Days StrapWire</t>
         </is>
       </c>
       <c r="E6" s="4" t="n">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>80Days CL101</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>80Days CL102</t>
         </is>
       </c>
       <c r="E8" s="4" t="n">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>80Days LD101</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Avento</t>
         </is>
       </c>
       <c r="E10" s="4" t="n">
@@ -4135,7 +4135,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Bowrider</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
@@ -4177,7 +4177,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Brentwood</t>
         </is>
       </c>
       <c r="E12" s="4" t="n">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux FX21</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Lantaka</t>
         </is>
       </c>
       <c r="E14" s="4" t="n">
@@ -4303,7 +4303,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Soleado</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
@@ -4345,7 +4345,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Sportech</t>
         </is>
       </c>
       <c r="E16" s="4" t="n">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Ventura</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
@@ -4429,7 +4429,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Sunglasses</t>
+          <t>Flux Verano</t>
         </is>
       </c>
       <c r="E18" s="4" t="n">

</xml_diff>

<commit_message>
Flux AU: complete portfolio cleanup — SP + SB all assigned
- 14 product-level portfolios created and assigned
- 7,449 SP + 1,283 SB = 8,732 total campaigns sorted
- 77 irrelevant SB campaigns paused + [ARCHIVE] prefixed
- Only 2 unmatched campaigns remain

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/flux/20260313_Flux_AU_Portfolio_Structure.xlsx
+++ b/flux/20260313_Flux_AU_Portfolio_Structure.xlsx
@@ -488,7 +488,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-13 11:25  |  Profile: 3601686309797276  |  SP+SB Campaigns: 8734</t>
+          <t>Generated: 2026-03-13 12:47  |  Profile: 3601686309797276  |  SP+SB Campaigns: 8734</t>
         </is>
       </c>
     </row>
@@ -567,13 +567,13 @@
         <v>532</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0</v>
+        <v>490</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>526</v>
+        <v>921</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6">
@@ -641,10 +641,10 @@
         <v>58</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>58</v>
+        <v>140</v>
       </c>
       <c r="I7" s="4" t="n">
         <v>0</v>
@@ -752,13 +752,13 @@
         <v>2622</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0</v>
+        <v>650</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>2486</v>
+        <v>3013</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>136</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11">
@@ -974,10 +974,10 @@
         <v>1255</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>1217</v>
+        <v>1220</v>
       </c>
       <c r="I16" s="4" t="n">
         <v>38</v>
@@ -1011,13 +1011,13 @@
         <v>771</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>341</v>
+        <v>383</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>430</v>
+        <v>446</v>
       </c>
     </row>
     <row r="18">
@@ -1070,19 +1070,19 @@
         <v>7449</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0</v>
+        <v>1283</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>6727</v>
+        <v>7776</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>722</v>
+        <v>956</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Unmatched campaigns: 1285</t>
+          <t>Unmatched campaigns: 2</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>532</v>
+        <v>1022</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>81</v>
@@ -3286,7 +3286,9 @@
       <c r="L4" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="M4" s="4" t="n"/>
+      <c r="M4" s="4" t="n">
+        <v>490</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -3336,7 +3338,7 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>58</v>
+        <v>140</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>58</v>
@@ -3348,7 +3350,9 @@
       <c r="J6" s="4" t="n"/>
       <c r="K6" s="4" t="n"/>
       <c r="L6" s="4" t="n"/>
-      <c r="M6" s="4" t="n"/>
+      <c r="M6" s="4" t="n">
+        <v>82</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -3431,7 +3435,7 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>2622</v>
+        <v>3272</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>339</v>
@@ -3457,7 +3461,9 @@
       <c r="L9" s="4" t="n">
         <v>2185</v>
       </c>
-      <c r="M9" s="4" t="n"/>
+      <c r="M9" s="4" t="n">
+        <v>650</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -3663,7 +3669,7 @@
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>1255</v>
+        <v>1258</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>327</v>
@@ -3685,7 +3691,9 @@
       <c r="L15" s="4" t="n">
         <v>790</v>
       </c>
-      <c r="M15" s="4" t="n"/>
+      <c r="M15" s="4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -3704,7 +3712,7 @@
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>771</v>
+        <v>829</v>
       </c>
       <c r="E16" s="4" t="n">
         <v>450</v>
@@ -3726,7 +3734,9 @@
       <c r="L16" s="4" t="n">
         <v>102</v>
       </c>
-      <c r="M16" s="4" t="n"/>
+      <c r="M16" s="4" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -3898,7 +3908,7 @@
         <v>532</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0</v>
+        <v>490</v>
       </c>
       <c r="I5" s="4" t="n">
         <v>8</v>
@@ -3982,7 +3992,7 @@
         <v>58</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="I7" s="4" t="n">
         <v>2</v>
@@ -4108,7 +4118,7 @@
         <v>2622</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0</v>
+        <v>650</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>6</v>
@@ -4360,7 +4370,7 @@
         <v>1255</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I16" s="4" t="n">
         <v>4</v>
@@ -4402,7 +4412,7 @@
         <v>771</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="I17" s="4" t="n">
         <v>6</v>

</xml_diff>